<commit_message>
Office tours grouped by type, Google 360 tours first
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,11 +36,15 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001C458C"/>
+    </font>
+    <font>
       <color rgb="001C458C"/>
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001C458C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE4F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,11 +74,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,7 +490,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -495,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -518,10 +528,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="63" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="39" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -538,374 +548,770 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>360 Virtual Clinic Tour</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>pinnaclechiropractic.net</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Google 360 tours (Street View inside the office) (18)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Virtual Tour of Facilities</t>
+          <t>Advanced Chiropractic &amp; Wellness Center, NJ</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>backpain631.com</t>
+          <t>drneilliebman.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Office Tour</t>
+          <t>California Oaks Chiropractic</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>rudinchiropractic.com</t>
+          <t>californiaoakschiropractic.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Take a Virtual Tour of Our Office</t>
+          <t>Chiropractor In White Plains, NY</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>kbchirohudson.com</t>
+          <t>drsutera.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>360 Virtual Reality Tour of Complete Care Chiropractic Office</t>
+          <t>Chiropractor in Denton, TX | Denton Chiropractic Center</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ccarechiro.com</t>
+          <t>dentonchiro.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Chiropractor in Excelsior, MN | Excelsior Chiropractic</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>integratedchirosd.com</t>
+          <t>excelsiorchiropractic.com</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Chiropractor in Jupiter, FL | La Ruffa Chiropractic &amp; Sports</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>downtownbroadwaychiro.com</t>
+          <t>drlaruffa.com</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Chiropractor in Mt. Airy, MD | Chiropractic First {PAGETITLE</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>drsutera.com</t>
+          <t>chiropractic-first.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chiropractor in Staten Island NY</t>
+          <t>Chiropractor in Setauket - East Setauket, NY | Setauket Chir</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>healthybodyny.com</t>
+          <t>setauketchiro.com</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Chiropractor in Stamford, CT | Stamford Sports &amp; Spine Stamf</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>evonchiro.com</t>
+          <t>stamfordsportsandspine.com</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Chiropractor in Rochester</t>
+          <t>Chiropractor in Trappe, PA | Swede Family Chiropractic</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>chiroroc.com</t>
+          <t>swedefamilychiropractic.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tour our Shelton Chiropractic Office</t>
+          <t>Chiropractor in Vernon Hills, IL | Molloy Chiropractic Cente</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>sheltonsportsandspine.com</t>
+          <t>molloychiropractic.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Chiropractors In New York, NY and Flushing, NY | Downtown Br</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>setauketchiro.com</t>
+          <t>downtownbroadwaychiro.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>KB Chiropractic</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>swedefamilychiropractic.com</t>
+          <t>kbchirohudson.com</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Not Acceptable!</t>
+          <t>Office Tour in Rochester | Chiropractic Associates of Roches</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>bexleychiropractic.com</t>
+          <t>chiroroc.com</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Pinnacle Chiropractic and Spinal Rehab Center of Highlands R</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>chiropractic-first.com</t>
+          <t>pinnaclechiropractic.net</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Office Tour</t>
+          <t>Prime Spine Plus</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>expeditionchiropractic.com</t>
+          <t>primespineplus.com (saved 2026)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Prohealth Chiropractic Rockville</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>stamfordsportsandspine.com</t>
+          <t>prohealthchiro.com</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>The Healthy Body | Staten Island Chiropractic :: Virtual Off</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>drlaruffa.com</t>
+          <t>healthybodyny.com</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Virtual Office Tour</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>molloychiropractic.com</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Other 360 degree virtual tours (1)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Virtual Office Tour</t>
+          <t>Complete Care Chiropractic</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>excelsiorchiropractic.com</t>
+          <t>ccarechiro.com</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Virtual Office Tour</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>dentonchiro.com</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>3D walk-through (Matterport) (1)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Not Acceptable!</t>
+          <t>Lakeshore Family Chiropractic</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>mnpainrelief.com</t>
+          <t>realitycaptureexperts.com</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>tampaholisticchiro.com</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>tampaholisticchiro.com (saved 2021)</t>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Video tours (1)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>gopremierchiro.com</t>
+          <t>Chiropractor in Yardley, PA | Evon Chiropractic</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>gopremierchiro.com (saved 2022)</t>
+          <t>evonchiro.com</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Office Tour</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>primespineplus.com (saved 2026)</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Photo tours (9)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Meet the Team</t>
+          <t>Bexley Chiropractor - Bexley Chiropractic Clinic</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>whiteoakchiropractic.com (saved 2026)</t>
+          <t>bexleychiropractic.com</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>drneilliebman.com</t>
+          <t>Chiropractor in Roseville, MN</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>drneilliebman.com</t>
+          <t>mnpainrelief.com</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sheppardspineandsports.com</t>
+          <t>Expedition Chiropractic</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>sheppardspineandsports.com</t>
+          <t>expeditionchiropractic.com</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>prohealthchiro.com</t>
+          <t>INTEGRATED CHIROPRACTIC AND REHAB</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>prohealthchiro.com</t>
+          <t>integratedchirosd.com</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>californiaoakschiropractic.com</t>
+          <t>Meet the Team</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>californiaoakschiropractic.com</t>
+          <t>whiteoakchiropractic.com (saved 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Office Tour</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>backpain631.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rudin Chiropractic</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>rudinchiropractic.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Shelton Sports and Spine | Shelton, CT Chiropractor | Dr. Ja</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>sheltonsportsandspine.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sheppard Spine &amp; Sports, Solana Beach</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>sheppardspineandsports.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saved pages (could not check) (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>gopremierchiro.com</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>gopremierchiro.com (saved 2022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>tampaholisticchiro.com</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>tampaholisticchiro.com (saved 2021)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId32"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Practice website</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Saved page</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>First saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>achiropracticwellnesscenter.com</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2009)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>alamedachiropractor.com</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2010)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>aligningwellness.com</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2011)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>backinbalance.com</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2008)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>backtoperformancechiro.com</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2011)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>baychirosantamonica.com</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2011)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>beneventochiro.com</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2009)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bestprosintown.com</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2025)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>bhchiro.com</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2014)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>chiropracticencinitas.com</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2014)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>chiropracticway.com</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2019)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>chiropractorbakersfield.com</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2019)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>chiropractoryubacity.com</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2019)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>cincinnatichiropractic.com</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2012)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>commonspirit.org</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2025)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>completebalancechiropractic.com</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2024)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2024</t>
         </is>
       </c>
     </row>
@@ -927,167 +1333,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId31"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="37" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Practice website</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Saved page</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>First saved</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>achiropracticwellnesscenter.com</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>saved office tour page (saved 2009)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>alamedachiropractor.com</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>saved office tour page (saved 2010)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>aligningwellness.com</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>saved office tour page (saved 2011)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>backinbalance.com</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>saved office tour page (saved 2008)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2008</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>backtoperformancechiro.com</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>saved office tour page (saved 2011)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>baychirosantamonica.com</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>saved office tour page (saved 2011)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Contra Costa: an interactive page (sortable table, map, CSV) for each list, plus every health discipline from the NPI registry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1312,6 +1312,40 @@
       <c r="C17" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>countryside-chiropractic.com</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2014)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>desalvochiropractic.com</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2019)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2019</t>
         </is>
       </c>
     </row>
@@ -1333,6 +1367,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Contra Costa pages: fill the filter dropdowns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1346,6 +1346,23 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>discovermhchiro.com</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2020)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2020</t>
         </is>
       </c>
     </row>
@@ -1369,6 +1386,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Interactive Contra Costa pages: CSV button only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1363,6 +1363,40 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>drderektaylor.com</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2020)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>drdewald.com</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2019)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2019</t>
         </is>
       </c>
     </row>
@@ -1387,6 +1421,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stop relying on the NPI registry: remove NPI-based pages and tables; home addresses from DCA + Assessor only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1397,6 +1397,23 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>drjoelchiropractic.com</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2015)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2015</t>
         </is>
       </c>
     </row>
@@ -1423,6 +1440,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Contra Costa: interactive pages for the rest of the county permits folder (massage inspections, vendors, Walnut Creek health businesses, home occupation, home wellness, STR, FBN)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1414,6 +1414,74 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>drpeterschiropractic.com</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2018)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>drpoller.com</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2025)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>dublinchiro.com</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2010)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>eilerchiro.com</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2019)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2019</t>
         </is>
       </c>
     </row>
@@ -1441,6 +1509,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Shared chiropractor buildings colored by license mix; no city-colored maps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/examples.xlsx
+++ b/downloads/examples.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1482,6 +1482,57 @@
       <c r="C27" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>fairwoodchiro.com</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2023)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>familyandsportschiropractic.com</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2016)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>feychiropractic.com</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>saved office tour page (saved 2008)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2008</t>
         </is>
       </c>
     </row>
@@ -1513,6 +1564,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>